<commit_message>
Sửa đường dẫn kết nối database với neon, sửa lại quản lí tạo lớp học ở lecturer
</commit_message>
<xml_diff>
--- a/Book1.xlsx
+++ b/Book1.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\NCKH\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/b5b7eb48b738fdcc/Documents/NCKH/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{84502C1B-046B-4881-911A-B0F60C515916}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="8" documentId="8_{84502C1B-046B-4881-911A-B0F60C515916}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F34C64A1-A52F-48BD-B013-C9485790B21E}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{BCDA0A0B-66CD-4AA6-AE4F-34937D8F078F}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{BCDA0A0B-66CD-4AA6-AE4F-34937D8F078F}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,12 +34,24 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2" uniqueCount="2">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
   <si>
     <t>Nguyễn Thị Diệu Hiền</t>
   </si>
   <si>
     <t>52400046@student.tdtu.edu.vn</t>
+  </si>
+  <si>
+    <t>Huỳnh Nguyễn Ngọc Thùy</t>
+  </si>
+  <si>
+    <t>52400319@student.tdtu.edu.vn</t>
+  </si>
+  <si>
+    <t>52400056@student.tdtu.edu.vn</t>
+  </si>
+  <si>
+    <t>Chu Đức Thành Nhân</t>
   </si>
 </sst>
 </file>
@@ -402,14 +414,14 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{447D020E-BE35-4204-A709-6EF15CEC04BA}">
-  <dimension ref="A1:D1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:D3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="18.44140625" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="27.21875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="18.453125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="27.1796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.35">
       <c r="A1">
         <v>52400046</v>
       </c>
@@ -420,12 +432,42 @@
         <v>1</v>
       </c>
       <c r="D1">
+        <v>24050302</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A2">
+        <v>52400319</v>
+      </c>
+      <c r="B2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="D2">
+        <v>24050402</v>
+      </c>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.35">
+      <c r="A3">
+        <v>52400056</v>
+      </c>
+      <c r="B3" t="s">
+        <v>5</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="D3">
         <v>24050302</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="C1" r:id="rId1" xr:uid="{2246FC30-5CE6-4CD0-97D8-74F21F294BE4}"/>
+    <hyperlink ref="C2" r:id="rId2" xr:uid="{AD63D198-D403-41A1-A980-82C918476EDF}"/>
+    <hyperlink ref="C3" r:id="rId3" xr:uid="{D01BDF17-D388-4819-952E-40BE4A824F2C}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>